<commit_message>
fix: close v0.2.1 five-table logic gaps
</commit_message>
<xml_diff>
--- a/config/new-five-tables/source/01_TCIM_十题_情境深描与条件边界表_V0.2.1_唯一运行版.xlsx
+++ b/config/new-five-tables/source/01_TCIM_十题_情境深描与条件边界表_V0.2.1_唯一运行版.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R810d42afb8194f7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RUNTIME_CONTRACT" sheetId="2" r:id="Rf4686d9298b24bdb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QUESTION_INDEX" sheetId="3" r:id="R531d62fa6cd34acb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DATA" sheetId="4" r:id="R329cb650d5054dda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DICTIONARY" sheetId="5" r:id="R3efff07dc42843a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ENUMS" sheetId="6" r:id="R4bedf4becdd247ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA_SUMMARY" sheetId="7" r:id="R8bf00cb9135c4067"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CHANGELOG" sheetId="8" r:id="Re3a256d3567146f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Ra09f7127ef0d4f43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RUNTIME_CONTRACT" sheetId="2" r:id="R4c3801621a5045c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QUESTION_INDEX" sheetId="3" r:id="R9459ef07faa84d23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DATA" sheetId="4" r:id="R7ce4d2ba68d649ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DICTIONARY" sheetId="5" r:id="Rd71722e7221b415e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ENUMS" sheetId="6" r:id="R94022039eaca4804"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA_SUMMARY" sheetId="7" r:id="Rb1c3600ac61640c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CHANGELOG" sheetId="8" r:id="R640dff19e8e0412c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15118,7 +15118,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e8bb589f279492f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3439f9476dfa4edd"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>